<commit_message>
Auto: PA-jobb uppdatering 2026-09-09
</commit_message>
<xml_diff>
--- a/PA_Jobb_Uppsala_Gunsta.xlsx
+++ b/PA_Jobb_Uppsala_Gunsta.xlsx
@@ -3102,7 +3102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M364"/>
+  <dimension ref="A1:M365"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3123,7 +3123,7 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="161" t="inlineStr">
         <is>
-          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-09-08 · 8 källor · Radie &lt;50 km · 0 nya · 1 borttagna</t>
+          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-09-09 · 8 källor · Radie &lt;50 km · 1 nya · 14 borttagna</t>
         </is>
       </c>
     </row>
@@ -25053,6 +25053,76 @@
           <t>🆕 NYTT
 2026-09-03
 🏛️ Platsbanken #31434238</t>
+        </is>
+      </c>
+    </row>
+    <row r="365" ht="55" customHeight="1">
+      <c r="A365" s="156" t="inlineStr">
+        <is>
+          <t>🆕 ⭐</t>
+        </is>
+      </c>
+      <c r="B365" s="133" t="inlineStr">
+        <is>
+          <t>Initiativrik assistent sökes till 8-årig kille</t>
+        </is>
+      </c>
+      <c r="C365" s="157" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D365" s="157" t="inlineStr">
+        <is>
+          <t>Östhammar</t>
+        </is>
+      </c>
+      <c r="E365" s="157" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F365" s="157" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="G365" s="158" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H365" s="158" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="I365" s="158" t="inlineStr">
+        <is>
+          <t>~49 km</t>
+        </is>
+      </c>
+      <c r="J365" s="157" t="inlineStr">
+        <is>
+          <t>– · ❓</t>
+        </is>
+      </c>
+      <c r="K365" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L365" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Behovsanst.</t>
+        </is>
+      </c>
+      <c r="M365" s="160" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-09-08
+🏛️ Platsbanken #31450097</t>
         </is>
       </c>
     </row>
@@ -25391,6 +25461,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B362" r:id="rId322"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B363" r:id="rId323"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B364" r:id="rId324"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B365" r:id="rId325"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto: PA-jobb uppdatering 2026-09-10
</commit_message>
<xml_diff>
--- a/PA_Jobb_Uppsala_Gunsta.xlsx
+++ b/PA_Jobb_Uppsala_Gunsta.xlsx
@@ -3102,7 +3102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M365"/>
+  <dimension ref="A1:M379"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3123,7 +3123,7 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="161" t="inlineStr">
         <is>
-          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-09-09 · 8 källor · Radie &lt;50 km · 1 nya · 14 borttagna</t>
+          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-09-10 · 8 källor · Radie &lt;50 km · 14 nya · 2 borttagna</t>
         </is>
       </c>
     </row>
@@ -25123,6 +25123,929 @@
           <t>🆕 NYTT
 2026-09-08
 🏛️ Platsbanken #31450097</t>
+        </is>
+      </c>
+    </row>
+    <row r="366" ht="55" customHeight="1">
+      <c r="A366" s="144" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐⭐</t>
+        </is>
+      </c>
+      <c r="B366" s="123" t="inlineStr">
+        <is>
+          <t>Personliga assistenter till en kille i Uppsala.</t>
+        </is>
+      </c>
+      <c r="C366" s="145" t="inlineStr">
+        <is>
+          <t>Inkludera assistans i Sverige AB</t>
+        </is>
+      </c>
+      <c r="D366" s="145" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E366" s="145" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F366" s="145" t="inlineStr">
+        <is>
+          <t>✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="G366" s="146" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H366" s="146" t="inlineStr"/>
+      <c r="I366" s="146" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J366" s="145" t="inlineStr">
+        <is>
+          <t>– · ✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="K366" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L366" s="159" t="inlineStr">
+        <is>
+          <t>🟡
+Kontrollera.</t>
+        </is>
+      </c>
+      <c r="M366" s="149" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-07-08
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="367" ht="55" customHeight="1">
+      <c r="A367" s="144" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐⭐</t>
+        </is>
+      </c>
+      <c r="B367" s="123" t="inlineStr">
+        <is>
+          <t>Söker dig som gillar ett aktivt jobb, som personlig assistent i Uppsala</t>
+        </is>
+      </c>
+      <c r="C367" s="145" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D367" s="145" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E367" s="145" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F367" s="145" t="inlineStr">
+        <is>
+          <t>✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="G367" s="146" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H367" s="146" t="inlineStr"/>
+      <c r="I367" s="146" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J367" s="145" t="inlineStr">
+        <is>
+          <t>– · ✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="K367" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L367" s="155" t="inlineStr">
+        <is>
+          <t>🔴
+Sommarvikariat.</t>
+        </is>
+      </c>
+      <c r="M367" s="149" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="368" ht="55" customHeight="1">
+      <c r="A368" s="144" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐⭐</t>
+        </is>
+      </c>
+      <c r="B368" s="123" t="inlineStr">
+        <is>
+          <t>Aktiv engagerad assistent sökes till kille i Tobo/Örbyhus, körkort krav</t>
+        </is>
+      </c>
+      <c r="C368" s="145" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D368" s="145" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E368" s="145" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F368" s="145" t="inlineStr">
+        <is>
+          <t>✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="G368" s="146" t="inlineStr">
+        <is>
+          <t>🚗 KRÄVS</t>
+        </is>
+      </c>
+      <c r="H368" s="146" t="inlineStr"/>
+      <c r="I368" s="146" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J368" s="145" t="inlineStr">
+        <is>
+          <t>🚗 KRÄVS · ✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="K368" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L368" s="155" t="inlineStr">
+        <is>
+          <t>🔴
+Sommarvikariat.</t>
+        </is>
+      </c>
+      <c r="M368" s="149" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-03-30
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="369" ht="55" customHeight="1">
+      <c r="A369" s="144" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐⭐</t>
+        </is>
+      </c>
+      <c r="B369" s="123" t="inlineStr">
+        <is>
+          <t>40% tjänst erbjudes till glad kille i Almunge</t>
+        </is>
+      </c>
+      <c r="C369" s="145" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D369" s="145" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E369" s="145" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F369" s="145" t="inlineStr">
+        <is>
+          <t>✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="G369" s="146" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H369" s="146" t="inlineStr"/>
+      <c r="I369" s="146" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J369" s="145" t="inlineStr">
+        <is>
+          <t>– · ✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="K369" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L369" s="159" t="inlineStr">
+        <is>
+          <t>🟡
+Kontrollera.</t>
+        </is>
+      </c>
+      <c r="M369" s="149" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-03-05
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="370" ht="55" customHeight="1">
+      <c r="A370" s="144" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐⭐</t>
+        </is>
+      </c>
+      <c r="B370" s="123" t="inlineStr">
+        <is>
+          <t>50% tjänst erbjudes till glad kille i Almunge</t>
+        </is>
+      </c>
+      <c r="C370" s="145" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D370" s="145" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E370" s="145" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F370" s="145" t="inlineStr">
+        <is>
+          <t>✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="G370" s="146" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H370" s="146" t="inlineStr"/>
+      <c r="I370" s="146" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J370" s="145" t="inlineStr">
+        <is>
+          <t>– · ✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="K370" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L370" s="159" t="inlineStr">
+        <is>
+          <t>🟡
+Kontrollera.</t>
+        </is>
+      </c>
+      <c r="M370" s="149" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-02-23
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="371" ht="55" customHeight="1">
+      <c r="A371" s="144" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐⭐</t>
+        </is>
+      </c>
+      <c r="B371" s="123" t="inlineStr">
+        <is>
+          <t>Har du barnasinnet kvar? Då har vi rätt jobb åt dig!</t>
+        </is>
+      </c>
+      <c r="C371" s="145" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D371" s="145" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E371" s="145" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F371" s="145" t="inlineStr">
+        <is>
+          <t>✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="G371" s="146" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H371" s="146" t="inlineStr"/>
+      <c r="I371" s="146" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J371" s="145" t="inlineStr">
+        <is>
+          <t>– · ✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="K371" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L371" s="159" t="inlineStr">
+        <is>
+          <t>🟡
+Kontrollera.</t>
+        </is>
+      </c>
+      <c r="M371" s="149" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-02-18
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="372" ht="55" customHeight="1">
+      <c r="A372" s="144" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐⭐</t>
+        </is>
+      </c>
+      <c r="B372" s="123" t="inlineStr">
+        <is>
+          <t>Personlig assistent till ung man i Uppsala</t>
+        </is>
+      </c>
+      <c r="C372" s="145" t="inlineStr">
+        <is>
+          <t>A-Assistans Leimir AB</t>
+        </is>
+      </c>
+      <c r="D372" s="145" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E372" s="145" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F372" s="145" t="inlineStr">
+        <is>
+          <t>✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="G372" s="146" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H372" s="146" t="inlineStr"/>
+      <c r="I372" s="146" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J372" s="145" t="inlineStr">
+        <is>
+          <t>– · ✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="K372" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L372" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Tills vidare.</t>
+        </is>
+      </c>
+      <c r="M372" s="149" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-02-13
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="373" ht="55" customHeight="1">
+      <c r="A373" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B373" s="129" t="inlineStr">
+        <is>
+          <t>Söker dig personlig assistent med intresse av matlagning och omvårdnad</t>
+        </is>
+      </c>
+      <c r="C373" s="152" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D373" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E373" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F373" s="152" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="G373" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H373" s="153" t="inlineStr"/>
+      <c r="I373" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J373" s="152" t="inlineStr">
+        <is>
+          <t>– · ❓</t>
+        </is>
+      </c>
+      <c r="K373" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L373" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Behovsanst.</t>
+        </is>
+      </c>
+      <c r="M373" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-04-17
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="374" ht="55" customHeight="1">
+      <c r="A374" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B374" s="129" t="inlineStr">
+        <is>
+          <t>Sommaren är räddad - Vi söker dig som vill jobba!</t>
+        </is>
+      </c>
+      <c r="C374" s="152" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D374" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E374" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F374" s="152" t="inlineStr">
+        <is>
+          <t>🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="G374" s="153" t="inlineStr">
+        <is>
+          <t>🚗 Merit</t>
+        </is>
+      </c>
+      <c r="H374" s="153" t="inlineStr"/>
+      <c r="I374" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J374" s="152" t="inlineStr">
+        <is>
+          <t>🚗 Merit · 🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="K374" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L374" s="155" t="inlineStr">
+        <is>
+          <t>🔴
+Sommarvikariat.</t>
+        </is>
+      </c>
+      <c r="M374" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-04-08
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="375" ht="55" customHeight="1">
+      <c r="A375" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B375" s="129" t="inlineStr">
+        <is>
+          <t>Engagerad assistent sökes till man i Enköping</t>
+        </is>
+      </c>
+      <c r="C375" s="152" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D375" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E375" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F375" s="152" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="G375" s="153" t="inlineStr">
+        <is>
+          <t>🚗 Merit</t>
+        </is>
+      </c>
+      <c r="H375" s="153" t="inlineStr"/>
+      <c r="I375" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J375" s="152" t="inlineStr">
+        <is>
+          <t>🚗 Merit · ❓</t>
+        </is>
+      </c>
+      <c r="K375" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L375" s="155" t="inlineStr">
+        <is>
+          <t>🔴
+Sommarvikariat.</t>
+        </is>
+      </c>
+      <c r="M375" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-03-30
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="376" ht="55" customHeight="1">
+      <c r="A376" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B376" s="129" t="inlineStr">
+        <is>
+          <t>Sommarvik med chans till förlängning  sökes till 29årig kille i Norrtälje</t>
+        </is>
+      </c>
+      <c r="C376" s="152" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D376" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E376" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F376" s="152" t="inlineStr">
+        <is>
+          <t>🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="G376" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H376" s="153" t="inlineStr"/>
+      <c r="I376" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J376" s="152" t="inlineStr">
+        <is>
+          <t>– · 🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="K376" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L376" s="155" t="inlineStr">
+        <is>
+          <t>🔴
+Sommarvikariat.</t>
+        </is>
+      </c>
+      <c r="M376" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-03-30
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="377" ht="55" customHeight="1">
+      <c r="A377" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B377" s="129" t="inlineStr">
+        <is>
+          <t>Extra jobb nu och i sommar? Vi söker Personliga assistenter!</t>
+        </is>
+      </c>
+      <c r="C377" s="152" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D377" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E377" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F377" s="152" t="inlineStr">
+        <is>
+          <t>🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="G377" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H377" s="153" t="inlineStr"/>
+      <c r="I377" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J377" s="152" t="inlineStr">
+        <is>
+          <t>– · 🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="K377" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L377" s="155" t="inlineStr">
+        <is>
+          <t>🔴
+Sommarvikariat.</t>
+        </is>
+      </c>
+      <c r="M377" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-03-30
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="378" ht="55" customHeight="1">
+      <c r="A378" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B378" s="129" t="inlineStr">
+        <is>
+          <t>Vi söker PA för kund i Stockholm</t>
+        </is>
+      </c>
+      <c r="C378" s="152" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D378" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E378" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F378" s="152" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="G378" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H378" s="153" t="inlineStr"/>
+      <c r="I378" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J378" s="152" t="inlineStr">
+        <is>
+          <t>– · ❓</t>
+        </is>
+      </c>
+      <c r="K378" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L378" s="159" t="inlineStr">
+        <is>
+          <t>🟡
+Kontrollera.</t>
+        </is>
+      </c>
+      <c r="M378" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-03-23
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="379" ht="55" customHeight="1">
+      <c r="A379" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B379" s="129" t="inlineStr">
+        <is>
+          <t>Vill du assistera mig på min gård utanför Uppsala?</t>
+        </is>
+      </c>
+      <c r="C379" s="152" t="inlineStr">
+        <is>
+          <t>Nära AB</t>
+        </is>
+      </c>
+      <c r="D379" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E379" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F379" s="152" t="inlineStr">
+        <is>
+          <t>🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="G379" s="153" t="inlineStr">
+        <is>
+          <t>🚗 Merit</t>
+        </is>
+      </c>
+      <c r="H379" s="153" t="inlineStr"/>
+      <c r="I379" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J379" s="152" t="inlineStr">
+        <is>
+          <t>🚗 Merit · 🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="K379" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L379" s="159" t="inlineStr">
+        <is>
+          <t>🟡
+Kontrollera.</t>
+        </is>
+      </c>
+      <c r="M379" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-02-19
+🟠 ledigajobbiuppsala.se</t>
         </is>
       </c>
     </row>
@@ -25462,6 +26385,20 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B363" r:id="rId323"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B364" r:id="rId324"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B365" r:id="rId325"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B366" r:id="rId326"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B367" r:id="rId327"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B368" r:id="rId328"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B369" r:id="rId329"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B370" r:id="rId330"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B371" r:id="rId331"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B372" r:id="rId332"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B373" r:id="rId333"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B374" r:id="rId334"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B375" r:id="rId335"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B376" r:id="rId336"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B377" r:id="rId337"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B378" r:id="rId338"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B379" r:id="rId339"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto: PA-jobb uppdatering 2026-09-11
</commit_message>
<xml_diff>
--- a/PA_Jobb_Uppsala_Gunsta.xlsx
+++ b/PA_Jobb_Uppsala_Gunsta.xlsx
@@ -3102,7 +3102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M379"/>
+  <dimension ref="A1:M380"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3123,7 +3123,7 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="161" t="inlineStr">
         <is>
-          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-09-10 · 8 källor · Radie &lt;50 km · 14 nya · 2 borttagna</t>
+          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-09-11 · 8 källor · Radie &lt;50 km · 1 nya · 1 borttagna</t>
         </is>
       </c>
     </row>
@@ -26046,6 +26046,67 @@
           <t>🆕 NYTT
 2026-02-19
 🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="380" ht="55" customHeight="1">
+      <c r="A380" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B380" s="129" t="inlineStr">
+        <is>
+          <t>NyMan i Uppsala söker assistans 15:00-21:00 mån-fre.</t>
+        </is>
+      </c>
+      <c r="C380" s="152" t="inlineStr"/>
+      <c r="D380" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E380" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F380" s="152" t="inlineStr">
+        <is>
+          <t>🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="G380" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H380" s="153" t="inlineStr"/>
+      <c r="I380" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J380" s="152" t="inlineStr">
+        <is>
+          <t>– · 🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="K380" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L380" s="159" t="inlineStr">
+        <is>
+          <t>🟡
+Kontrollera.</t>
+        </is>
+      </c>
+      <c r="M380" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+🔵 ledigajobb.se</t>
         </is>
       </c>
     </row>
@@ -26399,6 +26460,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B377" r:id="rId337"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B378" r:id="rId338"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B379" r:id="rId339"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B380" r:id="rId340"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto: PA-jobb uppdatering 2026-09-12
</commit_message>
<xml_diff>
--- a/PA_Jobb_Uppsala_Gunsta.xlsx
+++ b/PA_Jobb_Uppsala_Gunsta.xlsx
@@ -3102,7 +3102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M380"/>
+  <dimension ref="A1:M382"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3123,7 +3123,7 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="161" t="inlineStr">
         <is>
-          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-09-11 · 8 källor · Radie &lt;50 km · 1 nya · 1 borttagna</t>
+          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-09-12 · 8 källor · Radie &lt;50 km · 2 nya · 4 borttagna</t>
         </is>
       </c>
     </row>
@@ -26107,6 +26107,146 @@
         <is>
           <t>🆕 NYTT
 🔵 ledigajobb.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="381" ht="55" customHeight="1">
+      <c r="A381" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B381" s="129" t="inlineStr">
+        <is>
+          <t>Personlig assistent till man i Uppsala</t>
+        </is>
+      </c>
+      <c r="C381" s="152" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D381" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E381" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F381" s="152" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="G381" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H381" s="153" t="inlineStr">
+        <is>
+          <t>2027-03-10</t>
+        </is>
+      </c>
+      <c r="I381" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J381" s="152" t="inlineStr">
+        <is>
+          <t>– · ❓</t>
+        </is>
+      </c>
+      <c r="K381" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L381" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Behovsanst.</t>
+        </is>
+      </c>
+      <c r="M381" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-09-11
+🏛️ Platsbanken #31466858</t>
+        </is>
+      </c>
+    </row>
+    <row r="382" ht="55" customHeight="1">
+      <c r="A382" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B382" s="129" t="inlineStr">
+        <is>
+          <t>Man i Uppsala söker assistans 15:00-21:00 mån-fre.</t>
+        </is>
+      </c>
+      <c r="C382" s="152" t="inlineStr">
+        <is>
+          <t>God Assistans i Mitt AB</t>
+        </is>
+      </c>
+      <c r="D382" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E382" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F382" s="152" t="inlineStr">
+        <is>
+          <t>🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="G382" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H382" s="153" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="I382" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J382" s="152" t="inlineStr">
+        <is>
+          <t>– · 🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="K382" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L382" s="159" t="inlineStr">
+        <is>
+          <t>🟡
+Diskutera semester.</t>
+        </is>
+      </c>
+      <c r="M382" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-09-11
+🏛️ Platsbanken #31465008</t>
         </is>
       </c>
     </row>
@@ -26461,6 +26601,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B378" r:id="rId338"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B379" r:id="rId339"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B380" r:id="rId340"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B381" r:id="rId341"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B382" r:id="rId342"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto: PA-jobb uppdatering 2026-09-15
</commit_message>
<xml_diff>
--- a/PA_Jobb_Uppsala_Gunsta.xlsx
+++ b/PA_Jobb_Uppsala_Gunsta.xlsx
@@ -3102,7 +3102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M382"/>
+  <dimension ref="A1:M386"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3123,7 +3123,7 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="161" t="inlineStr">
         <is>
-          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-09-12 · 8 källor · Radie &lt;50 km · 2 nya · 4 borttagna</t>
+          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-09-15 · 8 källor · Radie &lt;50 km · 4 nya · 0 borttagna</t>
         </is>
       </c>
     </row>
@@ -26247,6 +26247,277 @@
           <t>🆕 NYTT
 2026-09-11
 🏛️ Platsbanken #31465008</t>
+        </is>
+      </c>
+    </row>
+    <row r="383" ht="55" customHeight="1">
+      <c r="A383" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B383" s="129" t="inlineStr">
+        <is>
+          <t>Timvikarier som personlig assistent sökes till en trevlig man i Uppsala</t>
+        </is>
+      </c>
+      <c r="C383" s="152" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D383" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E383" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F383" s="152" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="G383" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H383" s="153" t="inlineStr">
+        <is>
+          <t>2026-11-30</t>
+        </is>
+      </c>
+      <c r="I383" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J383" s="152" t="inlineStr">
+        <is>
+          <t>– · ❓</t>
+        </is>
+      </c>
+      <c r="K383" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L383" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Behovsanst.</t>
+        </is>
+      </c>
+      <c r="M383" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-09-15
+🏛️ Platsbanken #31477225</t>
+        </is>
+      </c>
+    </row>
+    <row r="384" ht="55" customHeight="1">
+      <c r="A384" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B384" s="129" t="inlineStr">
+        <is>
+          <t>Timvikarier sökes till man i Uppsala</t>
+        </is>
+      </c>
+      <c r="C384" s="152" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D384" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E384" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F384" s="152" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="G384" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H384" s="153" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="I384" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J384" s="152" t="inlineStr">
+        <is>
+          <t>– · ❓</t>
+        </is>
+      </c>
+      <c r="K384" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L384" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Behovsanst.</t>
+        </is>
+      </c>
+      <c r="M384" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-09-14
+🏛️ Platsbanken #31473263</t>
+        </is>
+      </c>
+    </row>
+    <row r="385" ht="55" customHeight="1">
+      <c r="A385" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B385" s="129" t="inlineStr">
+        <is>
+          <t>NyTimvikarier som personlig assistent sökes till en trevlig man i Uppsala</t>
+        </is>
+      </c>
+      <c r="C385" s="152" t="inlineStr"/>
+      <c r="D385" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E385" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F385" s="152" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="G385" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H385" s="153" t="inlineStr"/>
+      <c r="I385" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J385" s="152" t="inlineStr">
+        <is>
+          <t>– · ❓</t>
+        </is>
+      </c>
+      <c r="K385" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L385" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Behovsanst.</t>
+        </is>
+      </c>
+      <c r="M385" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+🔵 ledigajobb.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="386" ht="55" customHeight="1">
+      <c r="A386" s="156" t="inlineStr">
+        <is>
+          <t>🆕 ⭐</t>
+        </is>
+      </c>
+      <c r="B386" s="133" t="inlineStr">
+        <is>
+          <t>Personlig assistent timvikarie sökes till aktiv  man i Örbyhus</t>
+        </is>
+      </c>
+      <c r="C386" s="157" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D386" s="157" t="inlineStr">
+        <is>
+          <t>Tierp</t>
+        </is>
+      </c>
+      <c r="E386" s="157" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F386" s="157" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="G386" s="158" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H386" s="158" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="I386" s="158" t="inlineStr">
+        <is>
+          <t>~43 km</t>
+        </is>
+      </c>
+      <c r="J386" s="157" t="inlineStr">
+        <is>
+          <t>– · ❓</t>
+        </is>
+      </c>
+      <c r="K386" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L386" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Behovsanst.</t>
+        </is>
+      </c>
+      <c r="M386" s="160" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-09-14
+🏛️ Platsbanken #31471277</t>
         </is>
       </c>
     </row>
@@ -26603,6 +26874,10 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B380" r:id="rId340"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B381" r:id="rId341"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B382" r:id="rId342"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B383" r:id="rId343"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B384" r:id="rId344"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B385" r:id="rId345"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B386" r:id="rId346"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto: PA-jobb uppdatering 2026-09-22
</commit_message>
<xml_diff>
--- a/PA_Jobb_Uppsala_Gunsta.xlsx
+++ b/PA_Jobb_Uppsala_Gunsta.xlsx
@@ -3102,7 +3102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M386"/>
+  <dimension ref="A1:M388"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3123,7 +3123,7 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="161" t="inlineStr">
         <is>
-          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-09-21 · 8 källor · Radie &lt;50 km · 0 nya · 1 borttagna</t>
+          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-09-22 · 8 källor · Radie &lt;50 km · 2 nya · 0 borttagna</t>
         </is>
       </c>
     </row>
@@ -26518,6 +26518,137 @@
           <t>🆕 NYTT
 2026-09-14
 🏛️ Platsbanken #31471277</t>
+        </is>
+      </c>
+    </row>
+    <row r="387" ht="55" customHeight="1">
+      <c r="A387" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B387" s="129" t="inlineStr">
+        <is>
+          <t>Trygg och lyhörd assistent sökes till man i Uppsala – timanställning</t>
+        </is>
+      </c>
+      <c r="C387" s="152" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D387" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E387" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F387" s="152" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="G387" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H387" s="153" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="I387" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J387" s="152" t="inlineStr">
+        <is>
+          <t>– · ❓</t>
+        </is>
+      </c>
+      <c r="K387" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L387" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Behovsanst.</t>
+        </is>
+      </c>
+      <c r="M387" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-09-21
+🏛️ Platsbanken #31501050</t>
+        </is>
+      </c>
+    </row>
+    <row r="388" ht="55" customHeight="1">
+      <c r="A388" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B388" s="129" t="inlineStr">
+        <is>
+          <t>NyPersonlig assistent sökes till 18 årig pojke i Uppsala.</t>
+        </is>
+      </c>
+      <c r="C388" s="152" t="inlineStr"/>
+      <c r="D388" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E388" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F388" s="152" t="inlineStr">
+        <is>
+          <t>🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="G388" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H388" s="153" t="inlineStr"/>
+      <c r="I388" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J388" s="152" t="inlineStr">
+        <is>
+          <t>– · 🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="K388" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L388" s="159" t="inlineStr">
+        <is>
+          <t>🟡
+Kontrollera.</t>
+        </is>
+      </c>
+      <c r="M388" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+🔵 ledigajobb.se</t>
         </is>
       </c>
     </row>
@@ -26878,6 +27009,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B384" r:id="rId344"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B385" r:id="rId345"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B386" r:id="rId346"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B387" r:id="rId347"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B388" r:id="rId348"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto: PA-jobb uppdatering 2026-09-23
</commit_message>
<xml_diff>
--- a/PA_Jobb_Uppsala_Gunsta.xlsx
+++ b/PA_Jobb_Uppsala_Gunsta.xlsx
@@ -3102,7 +3102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M388"/>
+  <dimension ref="A1:M389"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3123,7 +3123,7 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="161" t="inlineStr">
         <is>
-          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-09-22 · 8 källor · Radie &lt;50 km · 2 nya · 0 borttagna</t>
+          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-09-23 · 8 källor · Radie &lt;50 km · 1 nya · 3 borttagna</t>
         </is>
       </c>
     </row>
@@ -26649,6 +26649,76 @@
         <is>
           <t>🆕 NYTT
 🔵 ledigajobb.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="389" ht="55" customHeight="1">
+      <c r="A389" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B389" s="129" t="inlineStr">
+        <is>
+          <t>Personlig assistent sökes till 18 årig pojke i Uppsala.</t>
+        </is>
+      </c>
+      <c r="C389" s="152" t="inlineStr">
+        <is>
+          <t>God Assistans i Mitt AB</t>
+        </is>
+      </c>
+      <c r="D389" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E389" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F389" s="152" t="inlineStr">
+        <is>
+          <t>🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="G389" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H389" s="153" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="I389" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J389" s="152" t="inlineStr">
+        <is>
+          <t>– · 🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="K389" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L389" s="159" t="inlineStr">
+        <is>
+          <t>🟡
+Diskutera semester.</t>
+        </is>
+      </c>
+      <c r="M389" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-09-22
+🏛️ Platsbanken #31503692</t>
         </is>
       </c>
     </row>
@@ -27011,6 +27081,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B386" r:id="rId346"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B387" r:id="rId347"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B388" r:id="rId348"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B389" r:id="rId349"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto: PA-jobb uppdatering 2026-09-29
</commit_message>
<xml_diff>
--- a/PA_Jobb_Uppsala_Gunsta.xlsx
+++ b/PA_Jobb_Uppsala_Gunsta.xlsx
@@ -3102,7 +3102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M389"/>
+  <dimension ref="A1:M391"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3123,7 +3123,7 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="161" t="inlineStr">
         <is>
-          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-09-26 · 8 källor · Radie &lt;50 km · 0 nya · 1 borttagna</t>
+          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-09-29 · 8 källor · Radie &lt;50 km · 2 nya · 0 borttagna</t>
         </is>
       </c>
     </row>
@@ -26719,6 +26719,146 @@
           <t>🆕 NYTT
 2026-09-22
 🏛️ Platsbanken #31503692</t>
+        </is>
+      </c>
+    </row>
+    <row r="390" ht="55" customHeight="1">
+      <c r="A390" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B390" s="129" t="inlineStr">
+        <is>
+          <t>Empatisk och engagerad assistent sökes till man</t>
+        </is>
+      </c>
+      <c r="C390" s="152" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D390" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E390" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F390" s="152" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="G390" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H390" s="153" t="inlineStr">
+        <is>
+          <t>2026-11-30</t>
+        </is>
+      </c>
+      <c r="I390" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J390" s="152" t="inlineStr">
+        <is>
+          <t>– · ❓</t>
+        </is>
+      </c>
+      <c r="K390" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L390" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Behovsanst.</t>
+        </is>
+      </c>
+      <c r="M390" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-09-28
+🏛️ Platsbanken #31528905</t>
+        </is>
+      </c>
+    </row>
+    <row r="391" ht="55" customHeight="1">
+      <c r="A391" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B391" s="129" t="inlineStr">
+        <is>
+          <t>Assistent med Manuellt körkort sökes till man</t>
+        </is>
+      </c>
+      <c r="C391" s="152" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D391" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E391" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F391" s="152" t="inlineStr">
+        <is>
+          <t>🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="G391" s="153" t="inlineStr">
+        <is>
+          <t>🚗 Merit</t>
+        </is>
+      </c>
+      <c r="H391" s="153" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="I391" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J391" s="152" t="inlineStr">
+        <is>
+          <t>🚗 Merit · 🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="K391" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L391" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Behovsanst.</t>
+        </is>
+      </c>
+      <c r="M391" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-09-28
+🏛️ Platsbanken #31527270</t>
         </is>
       </c>
     </row>
@@ -27082,6 +27222,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B387" r:id="rId347"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B388" r:id="rId348"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B389" r:id="rId349"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B390" r:id="rId350"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B391" r:id="rId351"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto: PA-jobb uppdatering 2026-10-06
</commit_message>
<xml_diff>
--- a/PA_Jobb_Uppsala_Gunsta.xlsx
+++ b/PA_Jobb_Uppsala_Gunsta.xlsx
@@ -3102,7 +3102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M391"/>
+  <dimension ref="A1:M392"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3123,7 +3123,7 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="161" t="inlineStr">
         <is>
-          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-10-05 · 8 källor · Radie &lt;50 km · 0 nya · 1 borttagna</t>
+          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-10-06 · 8 källor · Radie &lt;50 km · 1 nya · 0 borttagna</t>
         </is>
       </c>
     </row>
@@ -26859,6 +26859,76 @@
           <t>🆕 NYTT
 2026-09-28
 🏛️ Platsbanken #31527270</t>
+        </is>
+      </c>
+    </row>
+    <row r="392" ht="55" customHeight="1">
+      <c r="A392" s="156" t="inlineStr">
+        <is>
+          <t>🆕 ⭐</t>
+        </is>
+      </c>
+      <c r="B392" s="133" t="inlineStr">
+        <is>
+          <t>Musikintresserad man söker personliga assistenter i Heby</t>
+        </is>
+      </c>
+      <c r="C392" s="157" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D392" s="157" t="inlineStr">
+        <is>
+          <t>Heby</t>
+        </is>
+      </c>
+      <c r="E392" s="157" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F392" s="157" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="G392" s="158" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H392" s="158" t="inlineStr">
+        <is>
+          <t>2027-04-03</t>
+        </is>
+      </c>
+      <c r="I392" s="158" t="inlineStr">
+        <is>
+          <t>~47 km</t>
+        </is>
+      </c>
+      <c r="J392" s="157" t="inlineStr">
+        <is>
+          <t>– · ❓</t>
+        </is>
+      </c>
+      <c r="K392" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L392" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Behovsanst.</t>
+        </is>
+      </c>
+      <c r="M392" s="160" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-10-05
+🏛️ Platsbanken #31552166</t>
         </is>
       </c>
     </row>
@@ -27224,6 +27294,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B389" r:id="rId349"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B390" r:id="rId350"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B391" r:id="rId351"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B392" r:id="rId352"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto: PA-jobb uppdatering 2026-10-07
</commit_message>
<xml_diff>
--- a/PA_Jobb_Uppsala_Gunsta.xlsx
+++ b/PA_Jobb_Uppsala_Gunsta.xlsx
@@ -3102,7 +3102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M392"/>
+  <dimension ref="A1:M394"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3123,7 +3123,7 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="161" t="inlineStr">
         <is>
-          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-10-06 · 8 källor · Radie &lt;50 km · 1 nya · 0 borttagna</t>
+          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-10-07 · 8 källor · Radie &lt;50 km · 2 nya · 1 borttagna</t>
         </is>
       </c>
     </row>
@@ -26929,6 +26929,137 @@
           <t>🆕 NYTT
 2026-10-05
 🏛️ Platsbanken #31552166</t>
+        </is>
+      </c>
+    </row>
+    <row r="393" ht="55" customHeight="1">
+      <c r="A393" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B393" s="129" t="inlineStr">
+        <is>
+          <t>Timvikarie och engagerad assistent med bil, sökes till man i Enköping</t>
+        </is>
+      </c>
+      <c r="C393" s="152" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D393" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E393" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F393" s="152" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="G393" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H393" s="153" t="inlineStr">
+        <is>
+          <t>2026-12-15</t>
+        </is>
+      </c>
+      <c r="I393" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J393" s="152" t="inlineStr">
+        <is>
+          <t>– · ❓</t>
+        </is>
+      </c>
+      <c r="K393" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L393" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Behovsanst.</t>
+        </is>
+      </c>
+      <c r="M393" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-10-07
+🏛️ Platsbanken #31563912</t>
+        </is>
+      </c>
+    </row>
+    <row r="394" ht="55" customHeight="1">
+      <c r="A394" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B394" s="129" t="inlineStr">
+        <is>
+          <t>NyTimvikarie och engagerad assistent med bil, sökes till man i Enköping</t>
+        </is>
+      </c>
+      <c r="C394" s="152" t="inlineStr"/>
+      <c r="D394" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E394" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F394" s="152" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="G394" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H394" s="153" t="inlineStr"/>
+      <c r="I394" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J394" s="152" t="inlineStr">
+        <is>
+          <t>– · ❓</t>
+        </is>
+      </c>
+      <c r="K394" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L394" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Behovsanst.</t>
+        </is>
+      </c>
+      <c r="M394" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+🔵 ledigajobb.se</t>
         </is>
       </c>
     </row>
@@ -27295,6 +27426,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B390" r:id="rId350"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B391" r:id="rId351"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B392" r:id="rId352"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B393" r:id="rId353"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B394" r:id="rId354"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto: PA-jobb uppdatering 2026-10-08
</commit_message>
<xml_diff>
--- a/PA_Jobb_Uppsala_Gunsta.xlsx
+++ b/PA_Jobb_Uppsala_Gunsta.xlsx
@@ -3102,7 +3102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M394"/>
+  <dimension ref="A1:M395"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3123,7 +3123,7 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="161" t="inlineStr">
         <is>
-          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-10-07 · 8 källor · Radie &lt;50 km · 2 nya · 1 borttagna</t>
+          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-10-08 · 8 källor · Radie &lt;50 km · 1 nya · 1 borttagna</t>
         </is>
       </c>
     </row>
@@ -27060,6 +27060,76 @@
         <is>
           <t>🆕 NYTT
 🔵 ledigajobb.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="395" ht="55" customHeight="1">
+      <c r="A395" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B395" s="129" t="inlineStr">
+        <is>
+          <t>Avlösare i hemmet till sexårig pojke</t>
+        </is>
+      </c>
+      <c r="C395" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala kommun</t>
+        </is>
+      </c>
+      <c r="D395" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E395" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F395" s="152" t="inlineStr">
+        <is>
+          <t>🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="G395" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H395" s="153" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="I395" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J395" s="152" t="inlineStr">
+        <is>
+          <t>– · 🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="K395" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L395" s="159" t="inlineStr">
+        <is>
+          <t>🟡
+Diskutera semester.</t>
+        </is>
+      </c>
+      <c r="M395" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-10-07
+🏛️ Platsbanken #31566897</t>
         </is>
       </c>
     </row>
@@ -27428,6 +27498,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B392" r:id="rId352"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B393" r:id="rId353"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B394" r:id="rId354"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B395" r:id="rId355"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto: PA-jobb uppdatering 2026-10-09
</commit_message>
<xml_diff>
--- a/PA_Jobb_Uppsala_Gunsta.xlsx
+++ b/PA_Jobb_Uppsala_Gunsta.xlsx
@@ -3102,7 +3102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M395"/>
+  <dimension ref="A1:M396"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3123,7 +3123,7 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="161" t="inlineStr">
         <is>
-          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-10-08 · 8 källor · Radie &lt;50 km · 1 nya · 1 borttagna</t>
+          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-10-09 · 8 källor · Radie &lt;50 km · 1 nya · 1 borttagna</t>
         </is>
       </c>
     </row>
@@ -27130,6 +27130,76 @@
           <t>🆕 NYTT
 2026-10-07
 🏛️ Platsbanken #31566897</t>
+        </is>
+      </c>
+    </row>
+    <row r="396" ht="55" customHeight="1">
+      <c r="A396" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B396" s="129" t="inlineStr">
+        <is>
+          <t>Assistent sökes till 32-årig mjukvaruutvecklare i Uppsala, ca 70%</t>
+        </is>
+      </c>
+      <c r="C396" s="152" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D396" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E396" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F396" s="152" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="G396" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H396" s="153" t="inlineStr">
+        <is>
+          <t>2026-11-07</t>
+        </is>
+      </c>
+      <c r="I396" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J396" s="152" t="inlineStr">
+        <is>
+          <t>– · ❓</t>
+        </is>
+      </c>
+      <c r="K396" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L396" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Behovsanst.</t>
+        </is>
+      </c>
+      <c r="M396" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-10-08
+🏛️ Platsbanken #31571812</t>
         </is>
       </c>
     </row>
@@ -27499,6 +27569,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B393" r:id="rId353"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B394" r:id="rId354"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B395" r:id="rId355"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B396" r:id="rId356"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto: PA-jobb uppdatering 2026-10-10
</commit_message>
<xml_diff>
--- a/PA_Jobb_Uppsala_Gunsta.xlsx
+++ b/PA_Jobb_Uppsala_Gunsta.xlsx
@@ -3102,7 +3102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M396"/>
+  <dimension ref="A1:M397"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3123,7 +3123,7 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="161" t="inlineStr">
         <is>
-          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-10-09 · 8 källor · Radie &lt;50 km · 1 nya · 1 borttagna</t>
+          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-10-10 · 8 källor · Radie &lt;50 km · 1 nya · 1 borttagna</t>
         </is>
       </c>
     </row>
@@ -27200,6 +27200,76 @@
           <t>🆕 NYTT
 2026-10-08
 🏛️ Platsbanken #31571812</t>
+        </is>
+      </c>
+    </row>
+    <row r="397" ht="55" customHeight="1">
+      <c r="A397" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B397" s="129" t="inlineStr">
+        <is>
+          <t>Personliga assistenter sökes till man i 40-års åldern</t>
+        </is>
+      </c>
+      <c r="C397" s="152" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D397" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E397" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F397" s="152" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="G397" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H397" s="153" t="inlineStr">
+        <is>
+          <t>2026-11-30</t>
+        </is>
+      </c>
+      <c r="I397" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J397" s="152" t="inlineStr">
+        <is>
+          <t>– · ❓</t>
+        </is>
+      </c>
+      <c r="K397" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L397" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Behovsanst.</t>
+        </is>
+      </c>
+      <c r="M397" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-10-09
+🏛️ Platsbanken #31578374</t>
         </is>
       </c>
     </row>
@@ -27570,6 +27640,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B394" r:id="rId354"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B395" r:id="rId355"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B396" r:id="rId356"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B397" r:id="rId357"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto: PA-jobb uppdatering 2026-10-13
</commit_message>
<xml_diff>
--- a/PA_Jobb_Uppsala_Gunsta.xlsx
+++ b/PA_Jobb_Uppsala_Gunsta.xlsx
@@ -3102,7 +3102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M397"/>
+  <dimension ref="A1:M414"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3123,7 +3123,7 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="161" t="inlineStr">
         <is>
-          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-10-12 · 8 källor · Radie &lt;50 km · 0 nya · 15 borttagna</t>
+          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-10-13 · 8 källor · Radie &lt;50 km · 17 nya · 3 borttagna</t>
         </is>
       </c>
     </row>
@@ -27270,6 +27270,1131 @@
           <t>🆕 NYTT
 2026-10-09
 🏛️ Platsbanken #31578374</t>
+        </is>
+      </c>
+    </row>
+    <row r="398" ht="55" customHeight="1">
+      <c r="A398" s="144" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐⭐</t>
+        </is>
+      </c>
+      <c r="B398" s="123" t="inlineStr">
+        <is>
+          <t>Man i Uppsala söker assistans 15:00-21:00 mån-fre.</t>
+        </is>
+      </c>
+      <c r="C398" s="145" t="inlineStr">
+        <is>
+          <t>God Assistans i Mitt AB</t>
+        </is>
+      </c>
+      <c r="D398" s="145" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E398" s="145" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F398" s="145" t="inlineStr">
+        <is>
+          <t>✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="G398" s="146" t="inlineStr">
+        <is>
+          <t>🚗 Merit</t>
+        </is>
+      </c>
+      <c r="H398" s="146" t="inlineStr"/>
+      <c r="I398" s="146" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J398" s="145" t="inlineStr">
+        <is>
+          <t>🚗 Merit · ✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="K398" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L398" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Tills vidare.</t>
+        </is>
+      </c>
+      <c r="M398" s="149" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-09-11
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="399" ht="55" customHeight="1">
+      <c r="A399" s="144" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐⭐</t>
+        </is>
+      </c>
+      <c r="B399" s="123" t="inlineStr">
+        <is>
+          <t>Personliga assistenter till en kille i Uppsala.</t>
+        </is>
+      </c>
+      <c r="C399" s="145" t="inlineStr">
+        <is>
+          <t>Inkludera assistans i Sverige AB</t>
+        </is>
+      </c>
+      <c r="D399" s="145" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E399" s="145" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F399" s="145" t="inlineStr">
+        <is>
+          <t>✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="G399" s="146" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H399" s="146" t="inlineStr"/>
+      <c r="I399" s="146" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J399" s="145" t="inlineStr">
+        <is>
+          <t>– · ✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="K399" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L399" s="159" t="inlineStr">
+        <is>
+          <t>🟡
+Kontrollera.</t>
+        </is>
+      </c>
+      <c r="M399" s="149" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-07-08
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="400" ht="55" customHeight="1">
+      <c r="A400" s="144" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐⭐</t>
+        </is>
+      </c>
+      <c r="B400" s="123" t="inlineStr">
+        <is>
+          <t>Söker dig som gillar ett aktivt jobb, som personlig assistent i Uppsala</t>
+        </is>
+      </c>
+      <c r="C400" s="145" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D400" s="145" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E400" s="145" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F400" s="145" t="inlineStr">
+        <is>
+          <t>✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="G400" s="146" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H400" s="146" t="inlineStr"/>
+      <c r="I400" s="146" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J400" s="145" t="inlineStr">
+        <is>
+          <t>– · ✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="K400" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L400" s="155" t="inlineStr">
+        <is>
+          <t>🔴
+Sommarvikariat.</t>
+        </is>
+      </c>
+      <c r="M400" s="149" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="401" ht="55" customHeight="1">
+      <c r="A401" s="144" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐⭐</t>
+        </is>
+      </c>
+      <c r="B401" s="123" t="inlineStr">
+        <is>
+          <t>Aktiv engagerad assistent sökes till kille i Tobo/Örbyhus, körkort krav</t>
+        </is>
+      </c>
+      <c r="C401" s="145" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D401" s="145" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E401" s="145" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F401" s="145" t="inlineStr">
+        <is>
+          <t>✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="G401" s="146" t="inlineStr">
+        <is>
+          <t>🚗 KRÄVS</t>
+        </is>
+      </c>
+      <c r="H401" s="146" t="inlineStr"/>
+      <c r="I401" s="146" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J401" s="145" t="inlineStr">
+        <is>
+          <t>🚗 KRÄVS · ✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="K401" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L401" s="155" t="inlineStr">
+        <is>
+          <t>🔴
+Sommarvikariat.</t>
+        </is>
+      </c>
+      <c r="M401" s="149" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-03-30
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="402" ht="55" customHeight="1">
+      <c r="A402" s="144" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐⭐</t>
+        </is>
+      </c>
+      <c r="B402" s="123" t="inlineStr">
+        <is>
+          <t>40% tjänst erbjudes till glad kille i Almunge</t>
+        </is>
+      </c>
+      <c r="C402" s="145" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D402" s="145" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E402" s="145" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F402" s="145" t="inlineStr">
+        <is>
+          <t>✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="G402" s="146" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H402" s="146" t="inlineStr"/>
+      <c r="I402" s="146" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J402" s="145" t="inlineStr">
+        <is>
+          <t>– · ✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="K402" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L402" s="159" t="inlineStr">
+        <is>
+          <t>🟡
+Kontrollera.</t>
+        </is>
+      </c>
+      <c r="M402" s="149" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-03-05
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="403" ht="55" customHeight="1">
+      <c r="A403" s="144" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐⭐</t>
+        </is>
+      </c>
+      <c r="B403" s="123" t="inlineStr">
+        <is>
+          <t>50% tjänst erbjudes till glad kille i Almunge</t>
+        </is>
+      </c>
+      <c r="C403" s="145" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D403" s="145" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E403" s="145" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F403" s="145" t="inlineStr">
+        <is>
+          <t>✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="G403" s="146" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H403" s="146" t="inlineStr"/>
+      <c r="I403" s="146" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J403" s="145" t="inlineStr">
+        <is>
+          <t>– · ✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="K403" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L403" s="159" t="inlineStr">
+        <is>
+          <t>🟡
+Kontrollera.</t>
+        </is>
+      </c>
+      <c r="M403" s="149" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-02-23
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="404" ht="55" customHeight="1">
+      <c r="A404" s="144" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐⭐</t>
+        </is>
+      </c>
+      <c r="B404" s="123" t="inlineStr">
+        <is>
+          <t>Har du barnasinnet kvar? Då har vi rätt jobb åt dig!</t>
+        </is>
+      </c>
+      <c r="C404" s="145" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D404" s="145" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E404" s="145" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F404" s="145" t="inlineStr">
+        <is>
+          <t>✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="G404" s="146" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H404" s="146" t="inlineStr"/>
+      <c r="I404" s="146" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J404" s="145" t="inlineStr">
+        <is>
+          <t>– · ✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="K404" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L404" s="159" t="inlineStr">
+        <is>
+          <t>🟡
+Kontrollera.</t>
+        </is>
+      </c>
+      <c r="M404" s="149" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-02-18
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="405" ht="55" customHeight="1">
+      <c r="A405" s="144" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐⭐</t>
+        </is>
+      </c>
+      <c r="B405" s="123" t="inlineStr">
+        <is>
+          <t>Personlig assistent till ung man i Uppsala</t>
+        </is>
+      </c>
+      <c r="C405" s="145" t="inlineStr">
+        <is>
+          <t>A-Assistans Leimir AB</t>
+        </is>
+      </c>
+      <c r="D405" s="145" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E405" s="145" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F405" s="145" t="inlineStr">
+        <is>
+          <t>✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="G405" s="146" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H405" s="146" t="inlineStr"/>
+      <c r="I405" s="146" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J405" s="145" t="inlineStr">
+        <is>
+          <t>– · ✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="K405" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L405" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Tills vidare.</t>
+        </is>
+      </c>
+      <c r="M405" s="149" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-02-13
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="406" ht="55" customHeight="1">
+      <c r="A406" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B406" s="129" t="inlineStr">
+        <is>
+          <t>Personlig assistent till kille i Habo- dygnspass</t>
+        </is>
+      </c>
+      <c r="C406" s="152" t="inlineStr">
+        <is>
+          <t>Oberoende Liv i Jönköping, OLJA,                  Ekonomisk förening</t>
+        </is>
+      </c>
+      <c r="D406" s="152" t="inlineStr">
+        <is>
+          <t>Habo</t>
+        </is>
+      </c>
+      <c r="E406" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F406" s="152" t="inlineStr">
+        <is>
+          <t>🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="G406" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H406" s="153" t="inlineStr">
+        <is>
+          <t>2026-11-10</t>
+        </is>
+      </c>
+      <c r="I406" s="153" t="inlineStr">
+        <is>
+          <t>? km</t>
+        </is>
+      </c>
+      <c r="J406" s="152" t="inlineStr">
+        <is>
+          <t>– · 🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="K406" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L406" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Tills vidare.</t>
+        </is>
+      </c>
+      <c r="M406" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-10-12
+🏛️ Platsbanken #31585297</t>
+        </is>
+      </c>
+    </row>
+    <row r="407" ht="55" customHeight="1">
+      <c r="A407" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B407" s="129" t="inlineStr">
+        <is>
+          <t>Timvikarier sökes till social man i 70-års åldern i Uppsala</t>
+        </is>
+      </c>
+      <c r="C407" s="152" t="inlineStr">
+        <is>
+          <t>Alma assistans AB</t>
+        </is>
+      </c>
+      <c r="D407" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E407" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F407" s="152" t="inlineStr">
+        <is>
+          <t>🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="G407" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H407" s="153" t="inlineStr"/>
+      <c r="I407" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J407" s="152" t="inlineStr">
+        <is>
+          <t>– · 🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="K407" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L407" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Tills vidare.</t>
+        </is>
+      </c>
+      <c r="M407" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-08-26
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="408" ht="55" customHeight="1">
+      <c r="A408" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B408" s="129" t="inlineStr">
+        <is>
+          <t>Söker dig personlig assistent med intresse av matlagning och omvårdnad</t>
+        </is>
+      </c>
+      <c r="C408" s="152" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D408" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E408" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F408" s="152" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="G408" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H408" s="153" t="inlineStr"/>
+      <c r="I408" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J408" s="152" t="inlineStr">
+        <is>
+          <t>– · ❓</t>
+        </is>
+      </c>
+      <c r="K408" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L408" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Behovsanst.</t>
+        </is>
+      </c>
+      <c r="M408" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-04-17
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="409" ht="55" customHeight="1">
+      <c r="A409" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B409" s="129" t="inlineStr">
+        <is>
+          <t>Sommaren är räddad - Vi söker dig som vill jobba!</t>
+        </is>
+      </c>
+      <c r="C409" s="152" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D409" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E409" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F409" s="152" t="inlineStr">
+        <is>
+          <t>🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="G409" s="153" t="inlineStr">
+        <is>
+          <t>🚗 Merit</t>
+        </is>
+      </c>
+      <c r="H409" s="153" t="inlineStr"/>
+      <c r="I409" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J409" s="152" t="inlineStr">
+        <is>
+          <t>🚗 Merit · 🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="K409" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L409" s="155" t="inlineStr">
+        <is>
+          <t>🔴
+Sommarvikariat.</t>
+        </is>
+      </c>
+      <c r="M409" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-04-08
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="410" ht="55" customHeight="1">
+      <c r="A410" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B410" s="129" t="inlineStr">
+        <is>
+          <t>Sommarvik med chans till förlängning  sökes till 29årig kille i Norrtälje</t>
+        </is>
+      </c>
+      <c r="C410" s="152" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D410" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E410" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F410" s="152" t="inlineStr">
+        <is>
+          <t>🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="G410" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H410" s="153" t="inlineStr"/>
+      <c r="I410" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J410" s="152" t="inlineStr">
+        <is>
+          <t>– · 🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="K410" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L410" s="155" t="inlineStr">
+        <is>
+          <t>🔴
+Sommarvikariat.</t>
+        </is>
+      </c>
+      <c r="M410" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-03-30
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="411" ht="55" customHeight="1">
+      <c r="A411" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B411" s="129" t="inlineStr">
+        <is>
+          <t>Engagerad assistent sökes till man i Enköping</t>
+        </is>
+      </c>
+      <c r="C411" s="152" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D411" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E411" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F411" s="152" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="G411" s="153" t="inlineStr">
+        <is>
+          <t>🚗 Merit</t>
+        </is>
+      </c>
+      <c r="H411" s="153" t="inlineStr"/>
+      <c r="I411" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J411" s="152" t="inlineStr">
+        <is>
+          <t>🚗 Merit · ❓</t>
+        </is>
+      </c>
+      <c r="K411" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L411" s="155" t="inlineStr">
+        <is>
+          <t>🔴
+Sommarvikariat.</t>
+        </is>
+      </c>
+      <c r="M411" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-03-30
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="412" ht="55" customHeight="1">
+      <c r="A412" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B412" s="129" t="inlineStr">
+        <is>
+          <t>Extra jobb nu och i sommar? Vi söker Personliga assistenter!</t>
+        </is>
+      </c>
+      <c r="C412" s="152" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D412" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E412" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F412" s="152" t="inlineStr">
+        <is>
+          <t>🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="G412" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H412" s="153" t="inlineStr"/>
+      <c r="I412" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J412" s="152" t="inlineStr">
+        <is>
+          <t>– · 🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="K412" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L412" s="155" t="inlineStr">
+        <is>
+          <t>🔴
+Sommarvikariat.</t>
+        </is>
+      </c>
+      <c r="M412" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-03-30
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="413" ht="55" customHeight="1">
+      <c r="A413" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B413" s="129" t="inlineStr">
+        <is>
+          <t>Vi söker PA för kund i Stockholm</t>
+        </is>
+      </c>
+      <c r="C413" s="152" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D413" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E413" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F413" s="152" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="G413" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H413" s="153" t="inlineStr"/>
+      <c r="I413" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J413" s="152" t="inlineStr">
+        <is>
+          <t>– · ❓</t>
+        </is>
+      </c>
+      <c r="K413" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L413" s="159" t="inlineStr">
+        <is>
+          <t>🟡
+Kontrollera.</t>
+        </is>
+      </c>
+      <c r="M413" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-03-23
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="414" ht="55" customHeight="1">
+      <c r="A414" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B414" s="129" t="inlineStr">
+        <is>
+          <t>Vill du assistera mig på min gård utanför Uppsala?</t>
+        </is>
+      </c>
+      <c r="C414" s="152" t="inlineStr">
+        <is>
+          <t>Nära AB</t>
+        </is>
+      </c>
+      <c r="D414" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E414" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F414" s="152" t="inlineStr">
+        <is>
+          <t>🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="G414" s="153" t="inlineStr">
+        <is>
+          <t>🚗 Merit</t>
+        </is>
+      </c>
+      <c r="H414" s="153" t="inlineStr"/>
+      <c r="I414" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J414" s="152" t="inlineStr">
+        <is>
+          <t>🚗 Merit · 🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="K414" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L414" s="159" t="inlineStr">
+        <is>
+          <t>🟡
+Kontrollera.</t>
+        </is>
+      </c>
+      <c r="M414" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-02-19
+🟠 ledigajobbiuppsala.se</t>
         </is>
       </c>
     </row>
@@ -27641,6 +28766,23 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B395" r:id="rId355"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B396" r:id="rId356"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B397" r:id="rId357"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B398" r:id="rId358"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B399" r:id="rId359"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B400" r:id="rId360"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B401" r:id="rId361"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B402" r:id="rId362"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B403" r:id="rId363"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B404" r:id="rId364"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B405" r:id="rId365"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B406" r:id="rId366"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B407" r:id="rId367"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B408" r:id="rId368"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B409" r:id="rId369"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B410" r:id="rId370"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B411" r:id="rId371"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B412" r:id="rId372"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B413" r:id="rId373"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B414" r:id="rId374"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto: PA-jobb uppdatering 2026-10-16
</commit_message>
<xml_diff>
--- a/PA_Jobb_Uppsala_Gunsta.xlsx
+++ b/PA_Jobb_Uppsala_Gunsta.xlsx
@@ -3102,7 +3102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M414"/>
+  <dimension ref="A1:M415"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3123,7 +3123,7 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="161" t="inlineStr">
         <is>
-          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-10-13 · 8 källor · Radie &lt;50 km · 17 nya · 3 borttagna</t>
+          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-10-16 · 8 källor · Radie &lt;50 km · 1 nya · 1 borttagna</t>
         </is>
       </c>
     </row>
@@ -28395,6 +28395,76 @@
           <t>🆕 NYTT
 2026-02-19
 🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="415" ht="55" customHeight="1">
+      <c r="A415" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B415" s="129" t="inlineStr">
+        <is>
+          <t>Personliga assistenter sökes till en glad och nyfiken kille!</t>
+        </is>
+      </c>
+      <c r="C415" s="152" t="inlineStr">
+        <is>
+          <t>Inkludera Assistans AB</t>
+        </is>
+      </c>
+      <c r="D415" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E415" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F415" s="152" t="inlineStr">
+        <is>
+          <t>🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="G415" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H415" s="153" t="inlineStr">
+        <is>
+          <t>2026-12-31</t>
+        </is>
+      </c>
+      <c r="I415" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J415" s="152" t="inlineStr">
+        <is>
+          <t>– · 🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="K415" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L415" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Tills vidare.</t>
+        </is>
+      </c>
+      <c r="M415" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-10-15
+🏛️ Platsbanken #31600540</t>
         </is>
       </c>
     </row>
@@ -28783,6 +28853,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B412" r:id="rId372"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B413" r:id="rId373"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B414" r:id="rId374"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B415" r:id="rId375"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto: PA-jobb uppdatering 2026-10-17
</commit_message>
<xml_diff>
--- a/PA_Jobb_Uppsala_Gunsta.xlsx
+++ b/PA_Jobb_Uppsala_Gunsta.xlsx
@@ -3102,7 +3102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M415"/>
+  <dimension ref="A1:M416"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3123,7 +3123,7 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="161" t="inlineStr">
         <is>
-          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-10-16 · 8 källor · Radie &lt;50 km · 1 nya · 1 borttagna</t>
+          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-10-17 · 8 källor · Radie &lt;50 km · 1 nya · 1 borttagna</t>
         </is>
       </c>
     </row>
@@ -28465,6 +28465,76 @@
           <t>🆕 NYTT
 2026-10-15
 🏛️ Platsbanken #31600540</t>
+        </is>
+      </c>
+    </row>
+    <row r="416" ht="55" customHeight="1">
+      <c r="A416" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B416" s="129" t="inlineStr">
+        <is>
+          <t>Aktiv assistent sökes till aktiv ung man i Uppsala.</t>
+        </is>
+      </c>
+      <c r="C416" s="152" t="inlineStr">
+        <is>
+          <t>Särnmark Assistans AB</t>
+        </is>
+      </c>
+      <c r="D416" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E416" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F416" s="152" t="inlineStr">
+        <is>
+          <t>🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="G416" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H416" s="153" t="inlineStr">
+        <is>
+          <t>2026-11-14</t>
+        </is>
+      </c>
+      <c r="I416" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J416" s="152" t="inlineStr">
+        <is>
+          <t>– · 🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="K416" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L416" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Tills vidare.</t>
+        </is>
+      </c>
+      <c r="M416" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-10-16
+🏛️ Platsbanken #31608714</t>
         </is>
       </c>
     </row>
@@ -28854,6 +28924,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B413" r:id="rId373"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B414" r:id="rId374"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B415" r:id="rId375"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B416" r:id="rId376"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto: PA-jobb uppdatering 2026-10-19
</commit_message>
<xml_diff>
--- a/PA_Jobb_Uppsala_Gunsta.xlsx
+++ b/PA_Jobb_Uppsala_Gunsta.xlsx
@@ -3102,7 +3102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M416"/>
+  <dimension ref="A1:M417"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3123,7 +3123,7 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="161" t="inlineStr">
         <is>
-          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-10-17 · 8 källor · Radie &lt;50 km · 1 nya · 1 borttagna</t>
+          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-10-19 · 8 källor · Radie &lt;50 km · 1 nya · 0 borttagna</t>
         </is>
       </c>
     </row>
@@ -28535,6 +28535,72 @@
           <t>🆕 NYTT
 2026-10-16
 🏛️ Platsbanken #31608714</t>
+        </is>
+      </c>
+    </row>
+    <row r="417" ht="55" customHeight="1">
+      <c r="A417" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B417" s="129" t="inlineStr">
+        <is>
+          <t>Personlig assistent- Uppsala</t>
+        </is>
+      </c>
+      <c r="C417" s="152" t="inlineStr">
+        <is>
+          <t>Inova Assistans AB</t>
+        </is>
+      </c>
+      <c r="D417" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E417" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F417" s="152" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="G417" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H417" s="153" t="inlineStr"/>
+      <c r="I417" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J417" s="152" t="inlineStr">
+        <is>
+          <t>– · ❓</t>
+        </is>
+      </c>
+      <c r="K417" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L417" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Behovsanst.</t>
+        </is>
+      </c>
+      <c r="M417" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-03-31
+🟠 ledigajobbiuppsala.se</t>
         </is>
       </c>
     </row>
@@ -28925,6 +28991,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B414" r:id="rId374"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B415" r:id="rId375"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B416" r:id="rId376"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B417" r:id="rId377"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto: PA-jobb uppdatering 2026-10-20
</commit_message>
<xml_diff>
--- a/PA_Jobb_Uppsala_Gunsta.xlsx
+++ b/PA_Jobb_Uppsala_Gunsta.xlsx
@@ -3102,7 +3102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M417"/>
+  <dimension ref="A1:M419"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3123,7 +3123,7 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="161" t="inlineStr">
         <is>
-          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-10-19 · 8 källor · Radie &lt;50 km · 1 nya · 0 borttagna</t>
+          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-10-20 · 8 källor · Radie &lt;50 km · 2 nya · 0 borttagna</t>
         </is>
       </c>
     </row>
@@ -28601,6 +28601,146 @@
           <t>🆕 NYTT
 2026-03-31
 🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="418" ht="55" customHeight="1">
+      <c r="A418" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B418" s="129" t="inlineStr">
+        <is>
+          <t>Personliga assistenter sökes till man i Österbybruk – dag, kväll &amp; natt</t>
+        </is>
+      </c>
+      <c r="C418" s="152" t="inlineStr">
+        <is>
+          <t>Humana</t>
+        </is>
+      </c>
+      <c r="D418" s="152" t="inlineStr">
+        <is>
+          <t>Östhammar</t>
+        </is>
+      </c>
+      <c r="E418" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F418" s="152" t="inlineStr">
+        <is>
+          <t>🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="G418" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H418" s="153" t="inlineStr">
+        <is>
+          <t>2026-11-03</t>
+        </is>
+      </c>
+      <c r="I418" s="153" t="inlineStr">
+        <is>
+          <t>~49 km</t>
+        </is>
+      </c>
+      <c r="J418" s="152" t="inlineStr">
+        <is>
+          <t>– · 🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="K418" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L418" s="159" t="inlineStr">
+        <is>
+          <t>🟡
+Diskutera semester.</t>
+        </is>
+      </c>
+      <c r="M418" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-10-20
+🏛️ Platsbanken #31617476</t>
+        </is>
+      </c>
+    </row>
+    <row r="419" ht="55" customHeight="1">
+      <c r="A419" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B419" s="129" t="inlineStr">
+        <is>
+          <t>Trygg och lyhörd assistent sökes till man i Uppsala – timanställning</t>
+        </is>
+      </c>
+      <c r="C419" s="152" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D419" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E419" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F419" s="152" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="G419" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H419" s="153" t="inlineStr">
+        <is>
+          <t>2026-11-02</t>
+        </is>
+      </c>
+      <c r="I419" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J419" s="152" t="inlineStr">
+        <is>
+          <t>– · ❓</t>
+        </is>
+      </c>
+      <c r="K419" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L419" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Behovsanst.</t>
+        </is>
+      </c>
+      <c r="M419" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-10-20
+🏛️ Platsbanken #31617465</t>
         </is>
       </c>
     </row>
@@ -28992,6 +29132,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B415" r:id="rId375"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B416" r:id="rId376"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B417" r:id="rId377"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B418" r:id="rId378"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B419" r:id="rId379"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto: PA-jobb uppdatering 2026-10-21
</commit_message>
<xml_diff>
--- a/PA_Jobb_Uppsala_Gunsta.xlsx
+++ b/PA_Jobb_Uppsala_Gunsta.xlsx
@@ -3102,7 +3102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M419"/>
+  <dimension ref="A1:M420"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3123,7 +3123,7 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="161" t="inlineStr">
         <is>
-          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-10-20 · 8 källor · Radie &lt;50 km · 2 nya · 0 borttagna</t>
+          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-10-21 · 8 källor · Radie &lt;50 km · 1 nya · 0 borttagna</t>
         </is>
       </c>
     </row>
@@ -28741,6 +28741,76 @@
           <t>🆕 NYTT
 2026-10-20
 🏛️ Platsbanken #31617465</t>
+        </is>
+      </c>
+    </row>
+    <row r="420" ht="55" customHeight="1">
+      <c r="A420" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B420" s="129" t="inlineStr">
+        <is>
+          <t>Djur och bilintresserad kille söker en glad assistent</t>
+        </is>
+      </c>
+      <c r="C420" s="152" t="inlineStr">
+        <is>
+          <t>Vivida Assistans AB</t>
+        </is>
+      </c>
+      <c r="D420" s="152" t="inlineStr">
+        <is>
+          <t>Tierp</t>
+        </is>
+      </c>
+      <c r="E420" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F420" s="152" t="inlineStr">
+        <is>
+          <t>🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="G420" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H420" s="153" t="inlineStr">
+        <is>
+          <t>2026-11-30</t>
+        </is>
+      </c>
+      <c r="I420" s="153" t="inlineStr">
+        <is>
+          <t>~43 km</t>
+        </is>
+      </c>
+      <c r="J420" s="152" t="inlineStr">
+        <is>
+          <t>– · 🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="K420" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L420" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Tills vidare.</t>
+        </is>
+      </c>
+      <c r="M420" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-10-20
+🏛️ Platsbanken #31621958</t>
         </is>
       </c>
     </row>
@@ -29134,6 +29204,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B417" r:id="rId377"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B418" r:id="rId378"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B419" r:id="rId379"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B420" r:id="rId380"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto: PA-jobb uppdatering 2026-10-23
</commit_message>
<xml_diff>
--- a/PA_Jobb_Uppsala_Gunsta.xlsx
+++ b/PA_Jobb_Uppsala_Gunsta.xlsx
@@ -3102,7 +3102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M420"/>
+  <dimension ref="A1:M421"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3123,7 +3123,7 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="161" t="inlineStr">
         <is>
-          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-10-21 · 8 källor · Radie &lt;50 km · 1 nya · 0 borttagna</t>
+          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-10-23 · 8 källor · Radie &lt;50 km · 1 nya · 1 borttagna</t>
         </is>
       </c>
     </row>
@@ -28811,6 +28811,67 @@
           <t>🆕 NYTT
 2026-10-20
 🏛️ Platsbanken #31621958</t>
+        </is>
+      </c>
+    </row>
+    <row r="421" ht="55" customHeight="1">
+      <c r="A421" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B421" s="129" t="inlineStr">
+        <is>
+          <t>NySöker timvikarie till man i Uppsala, som lever ett aktivt liv</t>
+        </is>
+      </c>
+      <c r="C421" s="152" t="inlineStr"/>
+      <c r="D421" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E421" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F421" s="152" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="G421" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H421" s="153" t="inlineStr"/>
+      <c r="I421" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J421" s="152" t="inlineStr">
+        <is>
+          <t>– · ❓</t>
+        </is>
+      </c>
+      <c r="K421" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L421" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Behovsanst.</t>
+        </is>
+      </c>
+      <c r="M421" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+🔵 ledigajobb.se</t>
         </is>
       </c>
     </row>
@@ -29205,6 +29266,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B418" r:id="rId378"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B419" r:id="rId379"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B420" r:id="rId380"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B421" r:id="rId381"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto: PA-jobb uppdatering 2026-10-24
</commit_message>
<xml_diff>
--- a/PA_Jobb_Uppsala_Gunsta.xlsx
+++ b/PA_Jobb_Uppsala_Gunsta.xlsx
@@ -3102,7 +3102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M421"/>
+  <dimension ref="A1:M423"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3123,7 +3123,7 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="161" t="inlineStr">
         <is>
-          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-10-23 · 8 källor · Radie &lt;50 km · 1 nya · 1 borttagna</t>
+          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-10-24 · 8 källor · Radie &lt;50 km · 2 nya · 1 borttagna</t>
         </is>
       </c>
     </row>
@@ -28872,6 +28872,146 @@
         <is>
           <t>🆕 NYTT
 🔵 ledigajobb.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="422" ht="55" customHeight="1">
+      <c r="A422" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B422" s="129" t="inlineStr">
+        <is>
+          <t>Personlig assistent sökes till man vid Vaksalatorg</t>
+        </is>
+      </c>
+      <c r="C422" s="152" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D422" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E422" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F422" s="152" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="G422" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H422" s="153" t="inlineStr">
+        <is>
+          <t>2026-11-08</t>
+        </is>
+      </c>
+      <c r="I422" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J422" s="152" t="inlineStr">
+        <is>
+          <t>– · ❓</t>
+        </is>
+      </c>
+      <c r="K422" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L422" s="159" t="inlineStr">
+        <is>
+          <t>🟡
+Diskutera semester.</t>
+        </is>
+      </c>
+      <c r="M422" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-10-23
+🏛️ Platsbanken #31640318</t>
+        </is>
+      </c>
+    </row>
+    <row r="423" ht="55" customHeight="1">
+      <c r="A423" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B423" s="129" t="inlineStr">
+        <is>
+          <t>Söker timvikarie till man i Uppsala, som lever ett aktivt liv</t>
+        </is>
+      </c>
+      <c r="C423" s="152" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D423" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E423" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F423" s="152" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="G423" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H423" s="153" t="inlineStr">
+        <is>
+          <t>2026-12-15</t>
+        </is>
+      </c>
+      <c r="I423" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J423" s="152" t="inlineStr">
+        <is>
+          <t>– · ❓</t>
+        </is>
+      </c>
+      <c r="K423" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L423" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Behovsanst.</t>
+        </is>
+      </c>
+      <c r="M423" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-10-23
+🏛️ Platsbanken #31635144</t>
         </is>
       </c>
     </row>
@@ -29267,6 +29407,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B419" r:id="rId379"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B420" r:id="rId380"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B421" r:id="rId381"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B422" r:id="rId382"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B423" r:id="rId383"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>